<commit_message>
Fix: explicitly use n_last in PDF sheet slice computation
_local_function in writer.py was implicitly using n_first via the old
~-split. Now reads n directly as n_last, consistent across all three
sheets. Regenerated all 65 xlsx files.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workspaces/btc_daily_14days/cycle/cycle_phase.xlsx
+++ b/workspaces/btc_daily_14days/cycle/cycle_phase.xlsx
@@ -575,46 +575,46 @@
         <v>143</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>-5.640291467063122</v>
+        <v>-5.621626794213384</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>-6.554195988585676</v>
+        <v>-6.532985086416502</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>-10.44923052420802</v>
+        <v>-10.41481991172969</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>-15.92020532373565</v>
+        <v>-15.86770145192116</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-14.36317858438493</v>
+        <v>-14.31582471421817</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-18.27001143145282</v>
+        <v>-18.21010480397251</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>-16.95895467608668</v>
+        <v>-16.90294214693365</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>-16.73067372507044</v>
+        <v>-16.67553833671896</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>-16.79634530689784</v>
+        <v>-16.74051033666773</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>-15.5499624456874</v>
+        <v>-15.49831773085697</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>-12.95513509633809</v>
+        <v>-12.91174609239396</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>-15.72892001638123</v>
+        <v>-15.67651649984892</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>-13.3486757175037</v>
+        <v>-13.30420994935406</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>-6.787133218778926</v>
+        <v>-6.764202767074636</v>
       </c>
     </row>
     <row r="7">
@@ -627,46 +627,46 @@
         <v>142</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>4.548815200916785</v>
+        <v>4.534214841081649</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>4.346791186394633</v>
+        <v>4.332505561573335</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>4.657265258578207</v>
+        <v>4.642859172830676</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>9.017208522940564</v>
+        <v>8.988806383101576</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>14.1201887800944</v>
+        <v>14.07419154541006</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>10.89574692254573</v>
+        <v>10.86091742502042</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>12.92943417747281</v>
+        <v>12.88796227850231</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>11.75916164506616</v>
+        <v>11.72150418304309</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>10.28920579752404</v>
+        <v>10.25707656109713</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>12.96917190213077</v>
+        <v>12.92766381664815</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>9.942826784305282</v>
+        <v>9.911567007945322</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>9.979506820425769</v>
+        <v>9.948374348818959</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>8.854289028030031</v>
+        <v>8.826550244173937</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>6.28131408538821</v>
+        <v>6.261503920603573</v>
       </c>
     </row>
     <row r="8">
@@ -679,46 +679,46 @@
         <v>143</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>7.646421819650158</v>
+        <v>7.619744811650541</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>7.435473171109791</v>
+        <v>7.409166815417422</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>11.24035184338209</v>
+        <v>11.20156797561751</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>11.37362182142345</v>
+        <v>11.33469291269761</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>12.93808324452819</v>
+        <v>12.89269980709213</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>12.53892723862889</v>
+        <v>12.49559332389725</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>15.25915257168746</v>
+        <v>15.20623576096668</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>14.79517051070956</v>
+        <v>14.74386790274227</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>18.94247039397418</v>
+        <v>18.87727530483348</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>20.19877563249106</v>
+        <v>20.12850574954851</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>20.69982228310606</v>
+        <v>20.62813033013646</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>21.44101128287865</v>
+        <v>21.36696706557517</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>23.13015894227109</v>
+        <v>23.04982655627104</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>26.19464000223894</v>
+        <v>26.10293010005775</v>
       </c>
     </row>
     <row r="9">
@@ -731,46 +731,46 @@
         <v>142</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>8.774167313592685</v>
+        <v>8.741195807798185</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>9.277977298018619</v>
+        <v>9.242779264344257</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>13.1132597307646</v>
+        <v>13.06446704059424</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>16.06659563708229</v>
+        <v>16.00728126084461</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>13.41744185957673</v>
+        <v>13.36663972220686</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>15.83459713020071</v>
+        <v>15.77565850122242</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>15.04900395232904</v>
+        <v>14.9925956632352</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>16.70208632305714</v>
+        <v>16.6396411793725</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>18.76308524996262</v>
+        <v>18.6932962695203</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>21.44688391804257</v>
+        <v>21.3663645795298</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>26.19108036207126</v>
+        <v>26.09342896278456</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>28.35221798966907</v>
+        <v>28.2468058647827</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>31.47232575904231</v>
+        <v>31.35485938982865</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>30.31942584780023</v>
+        <v>30.20516589243439</v>
       </c>
     </row>
     <row r="10">
@@ -783,46 +783,46 @@
         <v>143</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>6.947121120349784</v>
+        <v>6.918379055144527</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>5.337321339904733</v>
+        <v>5.314261517149006</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>4.944001766819362</v>
+        <v>4.922402487619195</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>8.57565142069982</v>
+        <v>8.540048793897746</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>9.439871871399177</v>
+        <v>9.400039032997114</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>7.639654996358061</v>
+        <v>7.607156184257448</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5.455781258196659</v>
+        <v>5.431381081251509</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6.391119447407277</v>
+        <v>6.362924658299733</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4.22933153536065</v>
+        <v>4.209350727830532</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2.678265393656602</v>
+        <v>2.662873936504965</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4.578503886378158</v>
+        <v>4.555434940063705</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>6.018042454895529</v>
+        <v>5.98932503429905</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6.301328912669447</v>
+        <v>6.27041087691984</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>9.363299863096188</v>
+        <v>9.319713316841131</v>
       </c>
     </row>
     <row r="11">
@@ -835,46 +835,46 @@
         <v>142</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>2.436139144578441</v>
+        <v>2.422911002221284</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>11.39173685301393</v>
+        <v>11.3424533367914</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>9.591098580981892</v>
+        <v>9.549029420737156</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>11.13462694473838</v>
+        <v>11.08567455457483</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>8.48438808761739</v>
+        <v>8.444883948552437</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>10.19565047497373</v>
+        <v>10.15008582564309</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>8.703181271520457</v>
+        <v>8.663661091314921</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>8.943990570379817</v>
+        <v>8.903119631365847</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>4.650039567583207</v>
+        <v>4.626625877345511</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>3.800200409785027</v>
+        <v>3.778975090242142</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>2.184240010604299</v>
+        <v>2.168720504845062</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>2.220267897681957</v>
+        <v>2.204215484580452</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>1.800864496382005</v>
+        <v>1.785227640590179</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>-0.06681510958549097</v>
+        <v>-0.07652424841051442</v>
       </c>
     </row>
     <row r="12">
@@ -887,46 +887,46 @@
         <v>142</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1.027688440353565</v>
+        <v>1.019139740673246</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>1.529757060248691</v>
+        <v>1.517196765472313</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>7.477654425088154</v>
+        <v>7.44057791195555</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>4.086606286107539</v>
+        <v>4.062644825126092</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>5.664970403688606</v>
+        <v>5.633644159928132</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3.849019059856431</v>
+        <v>3.825822850393017</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3.765743857901803</v>
+        <v>3.74325356682801</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3.299492777659033</v>
+        <v>3.2784839365954</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>6.769483322529304</v>
+        <v>6.735072122053289</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>6.626623049142225</v>
+        <v>6.591644840511968</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>6.424315973677295</v>
+        <v>6.389655462401372</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4.341687727807809</v>
+        <v>4.315301763866174</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3.216093983802345</v>
+        <v>3.193113446216167</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>-0.06592476556651405</v>
+        <v>-0.07652424841051442</v>
       </c>
     </row>
     <row r="13">
@@ -939,46 +939,46 @@
         <v>144</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>-1.104549431321246</v>
+        <v>-1.10457683490457</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>-4.105852662667012</v>
+        <v>-4.094923179260249</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-4.501704325805328</v>
+        <v>-4.489850366582957</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>-2.286677753481939</v>
+        <v>-2.285015574991256</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>2.737460355883869</v>
+        <v>2.715944740884723</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.4413908746315087</v>
+        <v>-0.4480189070071745</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>5.736694303631708</v>
+        <v>5.703396669657458</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>1.790763089031323</v>
+        <v>1.774341219447287</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>2.426870108027835</v>
+        <v>2.408174473448767</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>1.576466482068085</v>
+        <v>1.560250332676894</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>3.463068789983055</v>
+        <v>3.438045266962206</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>3.499559334877851</v>
+        <v>3.474320128663976</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>1.686127838732411</v>
+        <v>1.667637229040963</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>1.939190903063391</v>
+        <v>1.918780915908734</v>
       </c>
     </row>
     <row r="14">
@@ -991,46 +991,46 @@
         <v>141</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1.407270899648346</v>
+        <v>1.395681912233592</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.5056239795014648</v>
+        <v>0.4964351288991367</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.1113066181805209</v>
+        <v>0.1031284485909865</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>5.922355716698753</v>
+        <v>5.886409500767016</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.4150999827897692</v>
+        <v>0.4021007340116824</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>2.8448244599563</v>
+        <v>2.822405351978112</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2.762068772864481</v>
+        <v>2.739100450825383</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3.717232503847193</v>
+        <v>3.690288745688157</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>8.636513967359761</v>
+        <v>8.587356872241024</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>7.788287290333152</v>
+        <v>7.741849805336862</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>8.298913615519183</v>
+        <v>8.249112150270605</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>9.761320524614064</v>
+        <v>9.70471987796239</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>10.05673968351332</v>
+        <v>9.997864019753159</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>10.31311818364873</v>
+        <v>10.25211424924206</v>
       </c>
     </row>
     <row r="15">
@@ -1043,46 +1043,46 @@
         <v>143</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>-1.444487271258922</v>
+        <v>-1.443480589846097</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>-1.657484331521779</v>
+        <v>-1.657161334819648</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>2.146384996296163</v>
+        <v>2.127476543679556</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>-0.5215078849268124</v>
+        <v>-0.5300262479513549</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>1.741709768087439</v>
+        <v>1.720903765446138</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>5.543820846203033</v>
+        <v>5.505945369959576</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>6.864020954329888</v>
+        <v>6.818737799398754</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>8.502373382519004</v>
+        <v>8.449382324307841</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>7.042938839340806</v>
+        <v>6.996300708297468</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>4.089351958262355</v>
+        <v>4.055926372438066</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>2.483538850360105</v>
+        <v>2.456651723596266</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>6.733590096892769</v>
+        <v>6.68567174401857</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>7.721041642297003</v>
+        <v>7.667252997935769</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>7.977253389951514</v>
+        <v>7.921111918239731</v>
       </c>
     </row>
     <row r="16">
@@ -1095,46 +1095,46 @@
         <v>143</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>5.548519721748221</v>
+        <v>5.513834721386786</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>6.037851415066697</v>
+        <v>5.998809706117676</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>7.045676797867152</v>
+        <v>6.999553453218638</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>8.580377128392456</v>
+        <v>8.524296434923428</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>5.244452689529531</v>
+        <v>5.203368555839205</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>2.742742866838093</v>
+        <v>2.714942864216844</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>4.062552132519436</v>
+        <v>4.026512030905359</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>2.194490421715237</v>
+        <v>2.167827459542671</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>0.7325824708471984</v>
+        <v>0.7130007113328674</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>1.986602882934683</v>
+        <v>1.960178486725148</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>0.3796803060007008</v>
+        <v>0.3605365596317824</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>-0.2852582076360903</v>
+        <v>-0.3026368287120462</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>-0.7047967052224635</v>
+        <v>-0.721502897346582</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>-3.262784277301392</v>
+        <v>-3.267699270571455</v>
       </c>
     </row>
     <row r="17">
@@ -1147,46 +1147,46 @@
         <v>141</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>-6.394147540068289</v>
+        <v>-6.368196954816035</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>-12.26531409706267</v>
+        <v>-12.20975476084194</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-11.24478777747364</v>
+        <v>-11.19721762354018</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>-16.0881421235345</v>
+        <v>-16.01713197741618</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-18.05333973383728</v>
+        <v>-17.97298791776321</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-20.60477620496739</v>
+        <v>-20.50929741393178</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>-22.11812944040587</v>
+        <v>-22.01650754385904</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>-26.86249248549989</v>
+        <v>-26.73478993618928</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>-31.20311225284352</v>
+        <v>-31.05188383233067</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>-30.64373953100377</v>
+        <v>-30.49639832135049</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>-31.57248232526</v>
+        <v>-31.4206747412547</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>-27.27335704439176</v>
+        <v>-27.14648639253448</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>-29.12969485562463</v>
+        <v>-28.99428298378209</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>-29.60148768755537</v>
+        <v>-29.46419780749552</v>
       </c>
     </row>
     <row r="18">
@@ -1199,46 +1199,46 @@
         <v>143</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>-3.542389369161022</v>
+        <v>-3.52961079721733</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>-7.254455016463055</v>
+        <v>-7.22078584279771</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>-10.45147317130454</v>
+        <v>-10.40248535269863</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>-13.82562771938275</v>
+        <v>-13.75871770885517</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>-15.77099845095246</v>
+        <v>-15.69368455989499</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-16.88146087819045</v>
+        <v>-16.79542205282861</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>-16.27105382514189</v>
+        <v>-16.19034162455046</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>-15.34405142136721</v>
+        <v>-15.26666914249083</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>-16.81572790427975</v>
+        <v>-16.72839621330348</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>-20.48361518133094</v>
+        <v>-20.3762902523892</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>-19.99490612183715</v>
+        <v>-19.89072387565321</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>-23.47925070036312</v>
+        <v>-23.35827455730661</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>-26.01922841957186</v>
+        <v>-25.88469419387798</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>-26.48121456696436</v>
+        <v>-26.34462234749469</v>
       </c>
     </row>
     <row r="19">
@@ -1251,46 +1251,46 @@
         <v>143</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>-2.143787970559465</v>
+        <v>-2.13788778242543</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>-3.057014116549496</v>
+        <v>-3.044622096307315</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-0.6530051083167479</v>
+        <v>-0.6576960627679966</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>-0.5221083259058901</v>
+        <v>-0.528024778022008</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-2.462300709431908</v>
+        <v>-2.456436296498069</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-2.86674931308761</v>
+        <v>-2.8553241933569</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>-3.652838547773918</v>
+        <v>-3.638865508752865</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>-4.825320170583566</v>
+        <v>-4.802205019785674</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>-2.081880833094921</v>
+        <v>-2.073414269157645</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>-1.531797425271499</v>
+        <v>-1.526593093465991</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>-1.737494178050795</v>
+        <v>-1.731583822425698</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>-0.9984024210111571</v>
+        <v>-0.9994205254534236</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>-2.124053381571592</v>
+        <v>-2.118383022802753</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>-5.390873007686395</v>
+        <v>-5.365601368473392</v>
       </c>
     </row>
     <row r="20">
@@ -1303,46 +1303,46 @@
         <v>142</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1.027688440353323</v>
+        <v>1.013513684465273</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>-4.811218881053705</v>
+        <v>-4.785458136086916</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-5.207904163334327</v>
+        <v>-5.183216048904342</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>-4.373930367806167</v>
+        <v>-4.355284638353197</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>-3.503778175483497</v>
+        <v>-3.490192663694614</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-4.620086876929633</v>
+        <v>-4.595438636664205</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>-8.23781373962693</v>
+        <v>-8.191563038871955</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>-7.29823423395618</v>
+        <v>-7.25545629087339</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>-10.19199969649679</v>
+        <v>-10.12878972344969</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>-10.34338129636589</v>
+        <v>-10.27927654583515</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>-11.26152927600445</v>
+        <v>-11.19191490635586</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>-15.47881772472304</v>
+        <v>-15.38442707831138</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>-15.90916495597842</v>
+        <v>-15.81170652476463</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>-14.95731312396295</v>
+        <v>-14.86525664277688</v>
       </c>
     </row>
     <row r="21">
@@ -1352,49 +1352,49 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>-7.717318917224986</v>
+        <v>-8.409451241299081</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>-12.66113937114937</v>
+        <v>-13.95416135247928</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-11.16700234830139</v>
+        <v>-12.23815585310152</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>-9.898920543759765</v>
+        <v>-10.81796726187655</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-13.00920114931689</v>
+        <v>-14.26757387293797</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-13.78990115237503</v>
+        <v>-15.20531164015444</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>-16.45781124380511</v>
+        <v>-18.14823643015561</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>-14.23940135740551</v>
+        <v>-15.73181613753574</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>-13.86228715645163</v>
+        <v>-15.35991690897056</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>-10.51168317608101</v>
+        <v>-11.64868447820862</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>-8.791347772799838</v>
+        <v>-9.741043550950785</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>-9.101477634942682</v>
+        <v>-10.06385469324278</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>-8.313077737931181</v>
+        <v>-9.198061811392932</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>-11.38942257354233</v>
+        <v>-12.61289952486243</v>
       </c>
     </row>
     <row r="22">
@@ -2213,10 +2213,8 @@
           <t>X &gt; 0.01924</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>4094~4107</t>
-        </is>
+      <c r="B6" t="n">
+        <v>4094</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>0.05099800801013998</v>
@@ -2267,10 +2265,8 @@
           <t>X &gt; 0.05235</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>3951~3964</t>
-        </is>
+      <c r="B7" t="n">
+        <v>3951</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>0.2563094093561205</v>
@@ -2321,10 +2317,8 @@
           <t>X &gt; 0.08546</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>3809~3822</t>
-        </is>
+      <c r="B8" t="n">
+        <v>3809</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>0.09682855577118943</v>
@@ -2375,10 +2369,8 @@
           <t>X &gt; 0.1186</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>3666~3679</t>
-        </is>
+      <c r="B9" t="n">
+        <v>3666</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>-0.1966185322241074</v>
@@ -2429,10 +2421,8 @@
           <t>X &gt; 0.1517</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>3524~3537</t>
-        </is>
+      <c r="B10" t="n">
+        <v>3524</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>-0.5567688262885682</v>
@@ -2483,10 +2473,8 @@
           <t>X &gt; 0.1848</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>3381~3394</t>
-        </is>
+      <c r="B11" t="n">
+        <v>3381</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>-0.8729315435452776</v>
@@ -2537,10 +2525,8 @@
           <t>X &gt; 0.2179</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>3239~3252</t>
-        </is>
+      <c r="B12" t="n">
+        <v>3239</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>-1.017423560062369</v>
@@ -2591,10 +2577,8 @@
           <t>X &gt; 0.251</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>3097~3110</t>
-        </is>
+      <c r="B13" t="n">
+        <v>3097</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>-1.110801664261423</v>
@@ -2645,10 +2629,8 @@
           <t>X &gt; 0.2841</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2953~2966</t>
-        </is>
+      <c r="B14" t="n">
+        <v>2953</v>
       </c>
       <c r="C14" s="4" t="n">
         <v>-1.111105211646247</v>
@@ -2699,10 +2681,8 @@
           <t>X &gt; 0.3172</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2812~2825</t>
-        </is>
+      <c r="B15" t="n">
+        <v>2812</v>
       </c>
       <c r="C15" s="4" t="n">
         <v>-1.236801152068381</v>
@@ -2753,10 +2733,8 @@
           <t>X &gt; 0.3503</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2669~2682</t>
-        </is>
+      <c r="B16" t="n">
+        <v>2669</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>-1.225727656526153</v>
@@ -2807,10 +2785,8 @@
           <t>X &gt; 0.3834</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2526~2539</t>
-        </is>
+      <c r="B17" t="n">
+        <v>2526</v>
       </c>
       <c r="C17" s="4" t="n">
         <v>-1.607262660501434</v>
@@ -2861,10 +2837,8 @@
           <t>X &gt; 0.4165</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2385~2398</t>
-        </is>
+      <c r="B18" t="n">
+        <v>2385</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>-1.325798620460183</v>
@@ -2915,10 +2889,8 @@
           <t>X &gt; 0.4496</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2242~2255</t>
-        </is>
+      <c r="B19" t="n">
+        <v>2242</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>-1.185234329079158</v>
@@ -2969,10 +2941,8 @@
           <t>X &gt; 0.4827</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2099~2112</t>
-        </is>
+      <c r="B20" t="n">
+        <v>2099</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>-1.12033225960392</v>
@@ -3023,10 +2993,8 @@
           <t>X &gt; 0.5159</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>1957~1970</t>
-        </is>
+      <c r="B21" t="n">
+        <v>1957</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>-1.275164208534854</v>
@@ -3077,10 +3045,8 @@
           <t>X &gt; 0.549</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>1836~1836</t>
-        </is>
+      <c r="B22" t="n">
+        <v>1836</v>
       </c>
       <c r="C22" s="4" t="n">
         <v>-0.804985161168581</v>
@@ -3131,10 +3097,8 @@
           <t>X &gt; 0.5821</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>1737~1737</t>
-        </is>
+      <c r="B23" t="n">
+        <v>1737</v>
       </c>
       <c r="C23" s="4" t="n">
         <v>-0.5072552459439947</v>
@@ -3185,10 +3149,8 @@
           <t>X &gt; 0.6152</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>1600~1600</t>
-        </is>
+      <c r="B24" t="n">
+        <v>1600</v>
       </c>
       <c r="C24" s="4" t="n">
         <v>-0.05593832020997525</v>
@@ -3239,10 +3201,8 @@
           <t>X &gt; 0.6483</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>1462~1462</t>
-        </is>
+      <c r="B25" t="n">
+        <v>1462</v>
       </c>
       <c r="C25" s="4" t="n">
         <v>0.03734143355199393</v>
@@ -3293,10 +3253,8 @@
           <t>X &gt; 0.6814</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>1324~1324</t>
-        </is>
+      <c r="B26" t="n">
+        <v>1324</v>
       </c>
       <c r="C26" s="4" t="n">
         <v>0.3766523142311158</v>
@@ -3347,10 +3305,8 @@
           <t>X &gt; 0.7145</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1187~1187</t>
-        </is>
+      <c r="B27" t="n">
+        <v>1187</v>
       </c>
       <c r="C27" s="4" t="n">
         <v>0.2445566250301212</v>
@@ -3401,10 +3357,8 @@
           <t>X &gt; 0.7476</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>1048~1048</t>
-        </is>
+      <c r="B28" t="n">
+        <v>1048</v>
       </c>
       <c r="C28" s="4" t="n">
         <v>0.08289755765261475</v>
@@ -3455,10 +3409,8 @@
           <t>X &gt; 0.7807</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>911~911</t>
-        </is>
+      <c r="B29" t="n">
+        <v>911</v>
       </c>
       <c r="C29" s="4" t="n">
         <v>0.1959140398339301</v>
@@ -3509,10 +3461,8 @@
           <t>X &gt; 0.8138</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>774~774</t>
-        </is>
+      <c r="B30" t="n">
+        <v>774</v>
       </c>
       <c r="C30" s="4" t="n">
         <v>-0.2970558912694088</v>
@@ -3563,10 +3513,8 @@
           <t>X &gt; 0.8469</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>635~635</t>
-        </is>
+      <c r="B31" t="n">
+        <v>635</v>
       </c>
       <c r="C31" s="4" t="n">
         <v>2.15223097112861</v>
@@ -3617,10 +3565,8 @@
           <t>X &gt; 0.88</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>498~498</t>
-        </is>
+      <c r="B32" t="n">
+        <v>498</v>
       </c>
       <c r="C32" s="4" t="n">
         <v>3.731461278183602</v>
@@ -3671,10 +3617,8 @@
           <t>X &gt; 0.9131</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>360~360</t>
-        </is>
+      <c r="B33" t="n">
+        <v>360</v>
       </c>
       <c r="C33" s="4" t="n">
         <v>4.173228346456689</v>
@@ -3725,10 +3669,8 @@
           <t>X &gt; 0.9462</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>222~222</t>
-        </is>
+      <c r="B34" t="n">
+        <v>222</v>
       </c>
       <c r="C34" s="4" t="n">
         <v>5.61466978789813</v>
@@ -3779,10 +3721,8 @@
           <t>X &gt; 0.9794</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>84~84</t>
-        </is>
+      <c r="B35" t="n">
+        <v>84</v>
       </c>
       <c r="C35" s="4" t="n">
         <v>3.458942632170981</v>
@@ -3967,10 +3907,8 @@
           <t>X &lt; 0.01924</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>84~84</t>
-        </is>
+      <c r="B6" t="n">
+        <v>84</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>-2.493438320209975</v>
@@ -4021,10 +3959,8 @@
           <t>X &lt; 0.05235</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>227~227</t>
-        </is>
+      <c r="B7" t="n">
+        <v>227</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>-4.475817174835527</v>
@@ -4075,10 +4011,8 @@
           <t>X &lt; 0.08546</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>369~369</t>
-        </is>
+      <c r="B8" t="n">
+        <v>369</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>-1.00292341506092</v>
@@ -4129,10 +4063,8 @@
           <t>X &lt; 0.1186</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>512~512</t>
-        </is>
+      <c r="B9" t="n">
+        <v>512</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>1.412811679790025</v>
@@ -4183,10 +4115,8 @@
           <t>X &lt; 0.1517</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>654~654</t>
-        </is>
+      <c r="B10" t="n">
+        <v>654</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>3.011148835753325</v>
@@ -4237,10 +4167,8 @@
           <t>X &lt; 0.1848</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>797~797</t>
-        </is>
+      <c r="B11" t="n">
+        <v>797</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>3.717352144030926</v>
@@ -4291,10 +4219,8 @@
           <t>X &lt; 0.2179</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>939~939</t>
-        </is>
+      <c r="B12" t="n">
+        <v>939</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>3.523601083410895</v>
@@ -4345,10 +4271,8 @@
           <t>X &lt; 0.251</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1081~1081</t>
-        </is>
+      <c r="B13" t="n">
+        <v>1081</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>3.195738368041646</v>
@@ -4399,10 +4323,8 @@
           <t>X &lt; 0.2841</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>1225~1225</t>
-        </is>
+      <c r="B14" t="n">
+        <v>1225</v>
       </c>
       <c r="C14" s="4" t="n">
         <v>2.690235149177774</v>
@@ -4453,10 +4375,8 @@
           <t>X &lt; 0.3172</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>1366~1366</t>
-        </is>
+      <c r="B15" t="n">
+        <v>1366</v>
       </c>
       <c r="C15" s="4" t="n">
         <v>2.557806189306866</v>
@@ -4507,10 +4427,8 @@
           <t>X &lt; 0.3503</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>1509~1509</t>
-        </is>
+      <c r="B16" t="n">
+        <v>1509</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>2.178529870644894</v>
@@ -4561,10 +4479,8 @@
           <t>X &lt; 0.3834</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>1652~1652</t>
-        </is>
+      <c r="B17" t="n">
+        <v>1652</v>
       </c>
       <c r="C17" s="4" t="n">
         <v>2.470242067199223</v>
@@ -4615,10 +4531,8 @@
           <t>X &lt; 0.4165</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>1793~1793</t>
-        </is>
+      <c r="B18" t="n">
+        <v>1793</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>1.773153983192145</v>
@@ -4669,10 +4583,8 @@
           <t>X &lt; 0.4496</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>1936~1936</t>
-        </is>
+      <c r="B19" t="n">
+        <v>1936</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>1.380528621938794</v>
@@ -4723,10 +4635,8 @@
           <t>X &lt; 0.4827</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2079~2079</t>
-        </is>
+      <c r="B20" t="n">
+        <v>2079</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>1.138115311343654</v>
@@ -4777,10 +4687,8 @@
           <t>X &lt; 0.5159</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2221~2221</t>
-        </is>
+      <c r="B21" t="n">
+        <v>2221</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>1.131055151199298</v>
@@ -4831,10 +4739,8 @@
           <t>X &lt; 0.549</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2342~2355</t>
-        </is>
+      <c r="B22" t="n">
+        <v>2342</v>
       </c>
       <c r="C22" s="4" t="n">
         <v>0.6275807880702757</v>
@@ -4885,10 +4791,8 @@
           <t>X &lt; 0.5821</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2441~2454</t>
-        </is>
+      <c r="B23" t="n">
+        <v>2441</v>
       </c>
       <c r="C23" s="4" t="n">
         <v>0.3590474173613316</v>
@@ -4939,10 +4843,8 @@
           <t>X &lt; 0.6152</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2578~2591</t>
-        </is>
+      <c r="B24" t="n">
+        <v>2578</v>
       </c>
       <c r="C24" s="4" t="n">
         <v>0.03454315412425046</v>
@@ -4993,10 +4895,8 @@
           <t>X &lt; 0.6483</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2716~2729</t>
-        </is>
+      <c r="B25" t="n">
+        <v>2716</v>
       </c>
       <c r="C25" s="4" t="n">
         <v>-0.02000482808831805</v>
@@ -5047,10 +4947,8 @@
           <t>X &lt; 0.6814</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2854~2867</t>
-        </is>
+      <c r="B26" t="n">
+        <v>2854</v>
       </c>
       <c r="C26" s="4" t="n">
         <v>-0.1739405873882163</v>
@@ -5101,10 +4999,8 @@
           <t>X &lt; 0.7145</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2991~3004</t>
-        </is>
+      <c r="B27" t="n">
+        <v>2991</v>
       </c>
       <c r="C27" s="4" t="n">
         <v>-0.09663405922461976</v>
@@ -5155,10 +5051,8 @@
           <t>X &lt; 0.7476</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>3130~3143</t>
-        </is>
+      <c r="B28" t="n">
+        <v>3130</v>
       </c>
       <c r="C28" s="4" t="n">
         <v>-0.02764131098312106</v>
@@ -5209,10 +5103,8 @@
           <t>X &lt; 0.7807</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>3267~3280</t>
-        </is>
+      <c r="B29" t="n">
+        <v>3267</v>
       </c>
       <c r="C29" s="4" t="n">
         <v>-0.05441392996607419</v>
@@ -5263,10 +5155,8 @@
           <t>X &lt; 0.8138</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>3404~3417</t>
-        </is>
+      <c r="B30" t="n">
+        <v>3404</v>
       </c>
       <c r="C30" s="4" t="n">
         <v>0.06728746264047203</v>
@@ -5317,10 +5207,8 @@
           <t>X &lt; 0.8469</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>3543~3556</t>
-        </is>
+      <c r="B31" t="n">
+        <v>3543</v>
       </c>
       <c r="C31" s="4" t="n">
         <v>-0.3843269591301137</v>
@@ -5371,10 +5259,8 @@
           <t>X &lt; 0.88</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>3680~3693</t>
-        </is>
+      <c r="B32" t="n">
+        <v>3680</v>
       </c>
       <c r="C32" s="4" t="n">
         <v>-0.5031864924276874</v>
@@ -5425,10 +5311,8 @@
           <t>X &lt; 0.9131</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>3818~3831</t>
-        </is>
+      <c r="B33" t="n">
+        <v>3818</v>
       </c>
       <c r="C33" s="4" t="n">
         <v>-0.3921592807946794</v>
@@ -5479,10 +5363,8 @@
           <t>X &lt; 0.9462</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>3956~3969</t>
-        </is>
+      <c r="B34" t="n">
+        <v>3956</v>
       </c>
       <c r="C34" s="4" t="n">
         <v>-0.3140480455816075</v>
@@ -5533,10 +5415,8 @@
           <t>X &lt; 0.9794</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>4094~4107</t>
-        </is>
+      <c r="B35" t="n">
+        <v>4094</v>
       </c>
       <c r="C35" s="4" t="n">
         <v>-0.07074535697646667</v>

</xml_diff>